<commit_message>
feat(catalog): add category provisioning import binding
</commit_message>
<xml_diff>
--- a/docs/operations/templates/ECIP_Stage0_Restaurant_Onboarding_v1.xlsx
+++ b/docs/operations/templates/ECIP_Stage0_Restaurant_Onboarding_v1.xlsx
@@ -51,7 +51,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'03_Resources'!$A$1:$E$501</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'04_Prep_Config'!$A$1:$B$501</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'05_Prep_Areas'!$A$1:$E$501</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'06_Categories'!$A$1:$E$501</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'06_Categories'!$A$1:$F$501</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'07_Products'!$A$1:$F$501</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'08_Product_Aliases'!$A$1:$D$501</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'08_Menus'!$A$1:$E$501</definedName>
@@ -1907,26 +1907,34 @@
       <text>
         <t>OBLIGATORIO
 Tipo: text
+Referencia inequívoca de la categoría Es una clave estable sólo dentro de este workbook; no es un ID de plataforma.
+Formato: ^[A-Z][A-Z0-9_-]{0,63}$</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>OBLIGATORIO
+Tipo: text
 Organización propietaria.
 Referencia: restaurant_profile.organization_code</t>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
+    <comment ref="C1" authorId="0" shapeId="0">
       <text>
         <t>OBLIGATORIO
 Tipo: text
 Nombre único dentro de la organización.</t>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>OPCIONAL
 Tipo: text
 Padre opcional en la misma organización.
-Referencia: categories.category_name</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
+Referencia: categories.category_key</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>OPCIONAL
 Tipo: integer
@@ -1934,7 +1942,7 @@
 Formato: &gt;=0</t>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>OBLIGATORIO
 Tipo: enum
@@ -1972,8 +1980,8 @@
       <text>
         <t>OPCIONAL
 Tipo: text
-Categoría opcional.
-Referencia: categories.category_name</t>
+Categoría elegida explícitamente; opcional.
+Referencia: categories.category_key</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
@@ -2746,7 +2754,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>organization_code + category_name</t>
+          <t>category_key</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3604,7 +3612,7 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -3623,7 +3631,7 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>category_name</t>
+          <t>category_key</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
@@ -6830,62 +6838,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
+          <t>category_key</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
           <t>organization_code</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>category_name</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>parent_category_name</t>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>name</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
+          <t>parent_category_key</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
           <t>display_order</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E501"/>
+  <autoFilter ref="A1:F501"/>
   <conditionalFormatting sqref="A2:A501">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND(COUNTA($A2:$E2)&gt;0,A2="")</formula>
+      <formula>AND(COUNTA($A2:$F2)&gt;0,A2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B501">
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>AND(COUNTA($A2:$E2)&gt;0,B2="")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E501">
+      <formula>AND(COUNTA($A2:$F2)&gt;0,B2="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C501">
     <cfRule type="expression" priority="3" dxfId="0">
-      <formula>AND(COUNTA($A2:$E2)&gt;0,E2="")</formula>
+      <formula>AND(COUNTA($A2:$F2)&gt;0,C2="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F501">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>AND(COUNTA($A2:$F2)&gt;0,F2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Valor no permitido" error="Seleccione un valor permitido por el contrato." promptTitle="Estado" prompt="Ciclo de vida del registro." type="list">
+    <dataValidation sqref="F2:F501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Valor no permitido" error="Seleccione un valor permitido por el contrato." promptTitle="Estado" prompt="Ciclo de vida del registro." type="list">
       <formula1>'_Lists'!$A$2:$A$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>